<commit_message>
feat: `x` in range mode will extend the range
</commit_message>
<xml_diff>
--- a/examples/test.xlsx
+++ b/examples/test.xlsx
@@ -60,31 +60,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:B3"/>
   <sheetData>
     <row r="1">
       <c r="A1">
-        <v>10</v>
+        <v>1</v>
       </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
-        <v>0</v>
+      <c r="B1">
+        <f>A1*2</f>
+        <v>2</v>
       </c>
     </row>
     <row r="2">
       <c r="A2">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>30</v>
-      </c>
-      <c r="B3">
-        <f>SUM(A1:A3)</f>
-        <v>50</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>